<commit_message>
docs: add troubleshooting log entries TR-004 to TR-007
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/troubleshooting.xlsx
+++ b/docs/troubleshooting.xlsx
@@ -118,7 +118,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -140,11 +140,80 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -182,6 +251,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,9 +626,9 @@
   <dimension ref="B2:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="32.16796875" customWidth="1"/>
-    <col min="3" max="3" width="40" customWidth="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="32.16796875" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
@@ -704,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -969,6 +1045,254 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>TR-004</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Frontend / CSS</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>globals.css에 남은 } 한 줄 때문에 모든 페이지가 빌드 오류 화면</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>개발 서버의 모든 경로에서 CssSyntaxError가 뜨고 화면이 오류 오버레이로 바뀜</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>정규식으로 CSS를 일괄 정리하다 닫는 중괄호 }가 하나 남음. eslint와 tsc는 CSS 문법을 검사하지 않아서 통과해 버림</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>lint와 tsc를 다시 돌렸지만 둘 다 통과해서 원인을 찾지 못함</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>남은 }를 제거하고 npm run build로 확인. 이후 CSS를 고치면 항상 빌드로 검증</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="inlineStr">
+        <is>
+          <t>반영 완료</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>- Always run `npm run build` after editing CSS; eslint and tsc do not parse CSS. (.claude/harness/rules/tailwind-v4.md)</t>
+        </is>
+      </c>
+      <c r="L5" s="9" t="inlineStr">
+        <is>
+          <t>Claude + 개발자</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>TR-005</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Frontend / 인증</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>docs 페이지를 열 때마다 POST /api/auth/refresh가 나가 콘솔에 500/401 에러</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>백엔드가 없는 환경에서 모든 docs 페이지의 콘솔에 빨간 에러가 쌓임</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>화면이 열릴 때마다 로그인 세션을 복원하려고 서버에 무조건 요청함</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>기록 없음</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>'이 브라우저에서 로그인한 적이 있음' 표시(localStorage의 meerkit-session)가 있을 때만 요청하고, 문서 전용 배포에서는 건너뜀. 이후 37개 페이지에서 /api 호출 0건 확인</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>반영 완료</t>
+        </is>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>- Never call /auth/refresh unconditionally on mount; gate it with the session hint. (.claude/harness/errors/next-app-router.md)</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Claude + 개발자</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>TR-006</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Frontend / docs 사이트</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>목차에서 항목이 두 개 동시에 활성화되고 React 같은 key 에러</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Pagination이 제목 id로 두 번 나와 목차 이중 활성화와 key 중복 에러가 생기고, 이전 페이지의 제목이 목차에 섞임</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>같은 이름의 소제목이 두 번 있어 id가 중복됨. Cache Components가 이전 페이지를 숨긴 채 남겨 두어, 전체 문서에서 제목을 찾으면 숨겨진 페이지의 제목까지 잡힘</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>기록 없음</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>목차와 앵커 조회를 현재 article 안으로 한정하고, 제목 id를 실행 중에 중복 제거하고, 겹치던 소제목 이름을 바꿈</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="inlineStr">
+        <is>
+          <t>반영 완료</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>- Always scope DOM queries (TOC, anchors) to the current article and de-duplicate heading ids at runtime. (.claude/harness/errors/next-app-router.md)</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>Claude + 개발자</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>TR-007</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Frontend / 애니메이션</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>'생각 중' 글자의 반짝임이 보이지 않음</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>반짝임 효과를 넣은 글자가 그냥 정지한 글자로 보임</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>한 요소에 animation을 가진 클래스 두 개(.mk-swap, .mk-shimmer-text)를 함께 붙여서 뒤의 animation이 앞의 것을 덮어씀</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>기록 없음</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>바깥 요소와 안쪽 요소로 나눠 각자 하나씩만 갖게 하고, 반짝이는 띠를 더 선명하게 바꿈</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>반영 완료</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>- Never put two animation-owning classes on one element; split into outer and inner elements. (.claude/harness/rules/tailwind-v4.md)</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Claude + 개발자</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -980,13 +1304,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D15"/>
+  <dimension ref="B2:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="59.61328125" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="59.61328125" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1114,23 +1438,21 @@
 7. 최종 해결책 (코드 변경점 포함) | 8. CLAUDE.md에 추가할 재발 방지 한 줄 규칙 (규칙 문체: Always/Never)</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="18" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
+      <c r="B16" s="21" t="n"/>
+      <c r="D16" s="22" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="D17" s="22" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="25" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>